<commit_message>
Enhance activity planning: multi-community support, delivery route synchronization, and UI improvements for journeys and planner
</commit_message>
<xml_diff>
--- a/Plantilla_Datos_Molinos_Guajira_V5.xlsx
+++ b/Plantilla_Datos_Molinos_Guajira_V5.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17580"/>
+    <workbookView windowHeight="17580" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="1. Molinos E Históricos" sheetId="1" r:id="rId1"/>
@@ -2533,7 +2533,10 @@
   <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="9" width="22" customWidth="1"/>
+    <col min="1" max="1" width="27.2857142857143" customWidth="1"/>
+    <col min="2" max="6" width="22" customWidth="1"/>
+    <col min="7" max="7" width="28" customWidth="1"/>
+    <col min="8" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" spans="1:9">
@@ -2578,7 +2581,9 @@
   <dimension ref="A1:G1"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="6"/>
   <cols>
-    <col min="1" max="7" width="22" customWidth="1"/>
+    <col min="1" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="27.2857142857143" customWidth="1"/>
+    <col min="6" max="7" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" spans="1:7">

</xml_diff>